<commit_message>
refactor: specific_param/parsing to update compute of columns min_stable_generation and add rounding to numeric columns for columns FO_ and PO_duration
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/thermal/specific_2030.xlsx
+++ b/tests/antares/resources/expected_output_files/thermal/specific_2030.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,207 +417,207 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>node</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Cluster</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>node_ENTSOE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>comments</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>cluster_PEMMDB</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>min_stable_gen</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>spinning</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>efficiency</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>FO_rate</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>FO_duration</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>PO_duration</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>PO_winter</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>marginal_cost</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>market_bid</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>MR_specific</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>CM_specific</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>nb_unit</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>F3</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>F5</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>F6</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>F7</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>F8</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>F9</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>F10</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>F11</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>F12</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>P9</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>P12</t>
         </is>
@@ -769,7 +757,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1.029878048780488</v>
+        <v>0.1416577903397606</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -888,7 +876,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1.940650406504065</v>
+        <v>0.5</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1126,7 +1114,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1.764836272040303</v>
+        <v>0.4</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -1245,7 +1233,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>0.3610718954248366</v>
+        <v>0.2</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1364,7 +1352,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>0.8755922865013775</v>
+        <v>0.1609316455696203</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -1602,7 +1590,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>0.4643990929705215</v>
+        <v>0.4</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -1840,7 +1828,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>2.759856630824373</v>
+        <v>0.6194690265486725</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -2078,7 +2066,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>0.6941573033707865</v>
+        <v>0.348056338028169</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -2197,7 +2185,7 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>1.496674057649667</v>
+        <v>0.3396910069951185</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -2316,7 +2304,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>0.7510384754125735</v>
+        <v>0.1990984060954279</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -2331,7 +2319,7 @@
         <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>27.00000000000001</v>
+        <v>27</v>
       </c>
       <c r="L16" t="n">
         <v>0.15</v>
@@ -2435,7 +2423,7 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>2.043902439024391</v>
+        <v>0.2364559819413093</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -2554,7 +2542,7 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>4.375</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -2673,7 +2661,7 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>0.9786407766990292</v>
+        <v>0.490272373540856</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -2792,7 +2780,7 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>1.375</v>
+        <v>0.360655737704918</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -2911,7 +2899,7 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>1.624761904761905</v>
+        <v>0.4335451080050826</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -3030,7 +3018,7 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>0.404</v>
+        <v>0.2082474226804124</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -3149,7 +3137,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>1.684210526315789</v>
+        <v>0.3437164339419979</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -3268,7 +3256,7 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>0.1590909090909091</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -3387,7 +3375,7 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>5.242574257425742</v>
+        <v>0.6723809523809524</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -3399,10 +3387,10 @@
         <v>0.06365714285714286</v>
       </c>
       <c r="J25" t="n">
-        <v>1.793650793650794</v>
+        <v>2</v>
       </c>
       <c r="K25" t="n">
-        <v>35.68571428571428</v>
+        <v>36</v>
       </c>
       <c r="L25" t="n">
         <v>0.005333333333333333</v>
@@ -3506,7 +3494,7 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -3518,7 +3506,7 @@
         <v>0.01</v>
       </c>
       <c r="J26" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="K26" t="n">
         <v>40</v>
@@ -3982,7 +3970,7 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
-        <v>0.9606557377049181</v>
+        <v>0.395945945945946</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -4101,7 +4089,7 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="n">
-        <v>1.536443481236455</v>
+        <v>0.5121478270788182</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
@@ -4220,7 +4208,7 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>2.708487084870849</v>
+        <v>0.6771217712177122</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
@@ -4339,7 +4327,7 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="n">
-        <v>1.401639344262295</v>
+        <v>0.4672131147540984</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
@@ -4458,7 +4446,7 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="n">
-        <v>0.8034433285509323</v>
+        <v>0.4017216642754661</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -4577,7 +4565,7 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
-        <v>5.079754601226994</v>
+        <v>0.8466257668711656</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -4696,7 +4684,7 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="n">
-        <v>0.4266666666666667</v>
+        <v>0.1066666666666667</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -4934,7 +4922,7 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="n">
-        <v>1.050639175257732</v>
+        <v>0.3244365210747485</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -5053,7 +5041,7 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="n">
-        <v>1.028169014084507</v>
+        <v>0.365</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -5172,7 +5160,7 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="n">
-        <v>1.438127090301003</v>
+        <v>0.4842342342342342</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
@@ -5291,7 +5279,7 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="n">
-        <v>0.370027183173378</v>
+        <v>0.2</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
@@ -5410,7 +5398,7 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="n">
-        <v>1.161247190572593</v>
+        <v>0.4466083399735535</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
@@ -5529,7 +5517,7 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="n">
-        <v>1.409122807017544</v>
+        <v>0.3673747778919421</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
@@ -5544,7 +5532,7 @@
         <v>7</v>
       </c>
       <c r="K43" t="n">
-        <v>54.00000000000001</v>
+        <v>54</v>
       </c>
       <c r="L43" t="n">
         <v>0.15</v>
@@ -5648,7 +5636,7 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="n">
-        <v>0.584</v>
+        <v>0.4</v>
       </c>
       <c r="G44" t="n">
         <v>0</v>
@@ -5767,7 +5755,7 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="n">
-        <v>0.8047910863509748</v>
+        <v>0.3902742131568283</v>
       </c>
       <c r="G45" t="n">
         <v>0</v>
@@ -5779,7 +5767,7 @@
         <v>0.04730000000000002</v>
       </c>
       <c r="J45" t="n">
-        <v>3.67</v>
+        <v>4</v>
       </c>
       <c r="K45" t="n">
         <v>70</v>
@@ -5886,7 +5874,7 @@
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="n">
-        <v>2.011358288770054</v>
+        <v>0.3172039927539411</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
@@ -5898,10 +5886,10 @@
         <v>0.04730000000000002</v>
       </c>
       <c r="J46" t="n">
-        <v>3.670000000000001</v>
+        <v>4</v>
       </c>
       <c r="K46" t="n">
-        <v>70.00000000000001</v>
+        <v>70</v>
       </c>
       <c r="L46" t="n">
         <v>0.4600000000000001</v>
@@ -6005,7 +5993,7 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="n">
-        <v>1.835602094240838</v>
+        <v>0.3491684095209641</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
@@ -6017,7 +6005,7 @@
         <v>0.04730000000000001</v>
       </c>
       <c r="J47" t="n">
-        <v>3.67</v>
+        <v>4</v>
       </c>
       <c r="K47" t="n">
         <v>70</v>
@@ -6124,7 +6112,7 @@
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="n">
-        <v>1.642764857881137</v>
+        <v>0.3905290186249938</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
@@ -6136,7 +6124,7 @@
         <v>0.0473</v>
       </c>
       <c r="J48" t="n">
-        <v>3.67</v>
+        <v>4</v>
       </c>
       <c r="K48" t="n">
         <v>70</v>
@@ -6243,7 +6231,7 @@
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="n">
-        <v>5.452000000000001</v>
+        <v>0.3744042632092187</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
@@ -6255,7 +6243,7 @@
         <v>0.04729999999999999</v>
       </c>
       <c r="J49" t="n">
-        <v>3.669999999999999</v>
+        <v>4</v>
       </c>
       <c r="K49" t="n">
         <v>70</v>
@@ -6362,7 +6350,7 @@
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="n">
-        <v>8.390182648401828</v>
+        <v>0.3833947477141749</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
@@ -6374,7 +6362,7 @@
         <v>0.04730000000000002</v>
       </c>
       <c r="J50" t="n">
-        <v>3.67</v>
+        <v>4</v>
       </c>
       <c r="K50" t="n">
         <v>70</v>
@@ -6481,7 +6469,7 @@
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="n">
-        <v>3.135324480069333</v>
+        <v>0.2466414609414088</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -6493,10 +6481,10 @@
         <v>0.06530650324021327</v>
       </c>
       <c r="J51" t="n">
-        <v>2.19974423084497</v>
+        <v>2</v>
       </c>
       <c r="K51" t="n">
-        <v>46.32172356791526</v>
+        <v>46</v>
       </c>
       <c r="L51" t="n">
         <v>0.2892961466524123</v>
@@ -6600,7 +6588,7 @@
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="n">
-        <v>2.440645687857078</v>
+        <v>0.3601846895074947</v>
       </c>
       <c r="G52" t="n">
         <v>0</v>
@@ -6612,7 +6600,7 @@
         <v>0.0473</v>
       </c>
       <c r="J52" t="n">
-        <v>3.67</v>
+        <v>4</v>
       </c>
       <c r="K52" t="n">
         <v>70</v>
@@ -6719,7 +6707,7 @@
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="n">
-        <v>1.374524714828897</v>
+        <v>0.2790966994788651</v>
       </c>
       <c r="G53" t="n">
         <v>0</v>
@@ -6731,7 +6719,7 @@
         <v>0.06379999999999998</v>
       </c>
       <c r="J53" t="n">
-        <v>2.25</v>
+        <v>2</v>
       </c>
       <c r="K53" t="n">
         <v>89</v>
@@ -6838,7 +6826,7 @@
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="n">
-        <v>1.144444444444444</v>
+        <v>0.3131841401118949</v>
       </c>
       <c r="G54" t="n">
         <v>0</v>
@@ -6850,7 +6838,7 @@
         <v>0.06380000000000001</v>
       </c>
       <c r="J54" t="n">
-        <v>2.25</v>
+        <v>2</v>
       </c>
       <c r="K54" t="n">
         <v>89</v>
@@ -6957,7 +6945,7 @@
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="n">
-        <v>0.7603501945525293</v>
+        <v>0.4164082893825582</v>
       </c>
       <c r="G55" t="n">
         <v>0</v>
@@ -6969,7 +6957,7 @@
         <v>0.0638</v>
       </c>
       <c r="J55" t="n">
-        <v>2.25</v>
+        <v>2</v>
       </c>
       <c r="K55" t="n">
         <v>89</v>
@@ -7076,7 +7064,7 @@
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="n">
-        <v>2.694411764705882</v>
+        <v>0.3136308392817405</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
@@ -7088,7 +7076,7 @@
         <v>0.03899999999999999</v>
       </c>
       <c r="J56" t="n">
-        <v>2.779999999999999</v>
+        <v>3</v>
       </c>
       <c r="K56" t="n">
         <v>36</v>
@@ -7195,7 +7183,7 @@
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="n">
-        <v>2.707584905660377</v>
+        <v>0.4516995154134409</v>
       </c>
       <c r="G57" t="n">
         <v>0</v>
@@ -7207,10 +7195,10 @@
         <v>0.0207</v>
       </c>
       <c r="J57" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="K57" t="n">
-        <v>58.99999999999999</v>
+        <v>59</v>
       </c>
       <c r="L57" t="n">
         <v>0.4099999999999999</v>
@@ -7314,7 +7302,7 @@
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="n">
-        <v>0.5571428571428571</v>
+        <v>0.3146112735706362</v>
       </c>
       <c r="G58" t="n">
         <v>0</v>
@@ -7326,10 +7314,10 @@
         <v>0.0207</v>
       </c>
       <c r="J58" t="n">
-        <v>0.9899999999999999</v>
+        <v>1</v>
       </c>
       <c r="K58" t="n">
-        <v>58.99999999999999</v>
+        <v>59</v>
       </c>
       <c r="L58" t="n">
         <v>0.41</v>
@@ -7433,7 +7421,7 @@
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="n">
-        <v>1.56887417218543</v>
+        <v>0.4465851037758969</v>
       </c>
       <c r="G59" t="n">
         <v>0</v>
@@ -7445,7 +7433,7 @@
         <v>0.0207</v>
       </c>
       <c r="J59" t="n">
-        <v>0.9900000000000001</v>
+        <v>1</v>
       </c>
       <c r="K59" t="n">
         <v>59</v>
@@ -7552,7 +7540,7 @@
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="n">
-        <v>1.406296851574213</v>
+        <v>0.4015926702915614</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
@@ -7564,7 +7552,7 @@
         <v>0.04730000000000001</v>
       </c>
       <c r="J60" t="n">
-        <v>3.67</v>
+        <v>4</v>
       </c>
       <c r="K60" t="n">
         <v>70</v>
@@ -7671,7 +7659,7 @@
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="n">
-        <v>3.08765</v>
+        <v>0.4142161466019157</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -7683,7 +7671,7 @@
         <v>0.04730000000000002</v>
       </c>
       <c r="J61" t="n">
-        <v>3.670000000000001</v>
+        <v>4</v>
       </c>
       <c r="K61" t="n">
         <v>70</v>
@@ -7790,7 +7778,7 @@
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="n">
-        <v>1.454330218068536</v>
+        <v>0.1833030995515977</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
@@ -7802,7 +7790,7 @@
         <v>0.0473</v>
       </c>
       <c r="J62" t="n">
-        <v>3.669999999999999</v>
+        <v>4</v>
       </c>
       <c r="K62" t="n">
         <v>70</v>
@@ -8266,7 +8254,7 @@
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="n">
-        <v>1.403573333333333</v>
+        <v>0.3907208076609012</v>
       </c>
       <c r="G66" t="n">
         <v>0</v>
@@ -8623,7 +8611,7 @@
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="n">
-        <v>0.2423076923076923</v>
+        <v>0.1148377688662049</v>
       </c>
       <c r="G69" t="n">
         <v>0</v>
@@ -8742,7 +8730,7 @@
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="n">
-        <v>0.7927272727272728</v>
+        <v>0.4</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
@@ -8861,7 +8849,7 @@
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="n">
-        <v>0.5384717607973423</v>
+        <v>0.4</v>
       </c>
       <c r="G71" t="n">
         <v>0</v>
@@ -8980,7 +8968,7 @@
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="n">
-        <v>1.597831637875121</v>
+        <v>0.6441778079144341</v>
       </c>
       <c r="G72" t="n">
         <v>0</v>
@@ -9218,7 +9206,7 @@
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="n">
-        <v>0.9986642920747997</v>
+        <v>0.5</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
@@ -9337,7 +9325,7 @@
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="n">
-        <v>0.9879226519337017</v>
+        <v>0.5</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
@@ -9456,7 +9444,7 @@
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="n">
-        <v>0.192</v>
+        <v>0.1826989619377163</v>
       </c>
       <c r="G76" t="n">
         <v>0</v>
@@ -9813,7 +9801,7 @@
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="n">
-        <v>2.068295081967213</v>
+        <v>0.3168839551847534</v>
       </c>
       <c r="G79" t="n">
         <v>0</v>
@@ -10051,7 +10039,7 @@
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="n">
-        <v>2.214</v>
+        <v>0.4438652766639936</v>
       </c>
       <c r="G81" t="n">
         <v>0</v>
@@ -10170,7 +10158,7 @@
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="n">
-        <v>0.8667278614442639</v>
+        <v>0.4</v>
       </c>
       <c r="G82" t="n">
         <v>0</v>
@@ -10289,7 +10277,7 @@
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="n">
-        <v>0.7456746499149326</v>
+        <v>0.4</v>
       </c>
       <c r="G83" t="n">
         <v>0</v>
@@ -10408,7 +10396,7 @@
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="n">
-        <v>3.070923076923077</v>
+        <v>1.568228210568039</v>
       </c>
       <c r="G84" t="n">
         <v>0</v>
@@ -10527,7 +10515,7 @@
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="n">
-        <v>0.6302421540392084</v>
+        <v>0.6134758535539871</v>
       </c>
       <c r="G85" t="n">
         <v>0</v>
@@ -11122,7 +11110,7 @@
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="n">
-        <v>23.53484398915174</v>
+        <v>0.5</v>
       </c>
       <c r="G90" t="n">
         <v>0</v>
@@ -11241,7 +11229,7 @@
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="n">
-        <v>8.862747380675204</v>
+        <v>0.3099841854359429</v>
       </c>
       <c r="G91" t="n">
         <v>0</v>
@@ -11360,7 +11348,7 @@
       <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="n">
-        <v>3.081116646301344</v>
+        <v>0.6427324954412658</v>
       </c>
       <c r="G92" t="n">
         <v>0</v>
@@ -11372,7 +11360,7 @@
         <v>0.05</v>
       </c>
       <c r="J92" t="n">
-        <v>6.999999999999999</v>
+        <v>7</v>
       </c>
       <c r="K92" t="n">
         <v>54</v>
@@ -11479,7 +11467,7 @@
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="G93" t="n">
         <v>0</v>
@@ -11494,7 +11482,7 @@
         <v>2</v>
       </c>
       <c r="K93" t="n">
-        <v>97.5</v>
+        <v>98</v>
       </c>
       <c r="L93" t="n">
         <v>0.0375</v>
@@ -11717,7 +11705,7 @@
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="n">
-        <v>0.7038461538461539</v>
+        <v>0.2534626038781164</v>
       </c>
       <c r="G95" t="n">
         <v>0</v>
@@ -11732,7 +11720,7 @@
         <v>2</v>
       </c>
       <c r="K95" t="n">
-        <v>41.71745152354571</v>
+        <v>42</v>
       </c>
       <c r="L95" t="n">
         <v>0</v>
@@ -11836,7 +11824,7 @@
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="n">
-        <v>1.709316770186335</v>
+        <v>0.8311688311688311</v>
       </c>
       <c r="G96" t="n">
         <v>0</v>
@@ -11851,7 +11839,7 @@
         <v>2</v>
       </c>
       <c r="K96" t="n">
-        <v>53.40380549682875</v>
+        <v>53</v>
       </c>
       <c r="L96" t="n">
         <v>0</v>
@@ -11955,7 +11943,7 @@
       <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="n">
-        <v>1.935714285714286</v>
+        <v>0.6678989525569933</v>
       </c>
       <c r="G97" t="n">
         <v>0</v>
@@ -11970,7 +11958,7 @@
         <v>2</v>
       </c>
       <c r="K97" t="n">
-        <v>68.55206407886629</v>
+        <v>69</v>
       </c>
       <c r="L97" t="n">
         <v>0</v>
@@ -12074,7 +12062,7 @@
       <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="n">
-        <v>0.9600000000000001</v>
+        <v>0.4</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -12089,7 +12077,7 @@
         <v>2</v>
       </c>
       <c r="K98" t="n">
-        <v>92.5</v>
+        <v>92</v>
       </c>
       <c r="L98" t="n">
         <v>0</v>
@@ -12193,7 +12181,7 @@
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="n">
-        <v>1.816</v>
+        <v>0.6355205599300088</v>
       </c>
       <c r="G99" t="n">
         <v>0</v>
@@ -12205,10 +12193,10 @@
         <v>0.030498687664042</v>
       </c>
       <c r="J99" t="n">
-        <v>3.099737532808399</v>
+        <v>3</v>
       </c>
       <c r="K99" t="n">
-        <v>23.21084864391951</v>
+        <v>23</v>
       </c>
       <c r="L99" t="n">
         <v>0</v>
@@ -12312,7 +12300,7 @@
       <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="n">
-        <v>0.3984</v>
+        <v>0.2316279069767442</v>
       </c>
       <c r="G100" t="n">
         <v>0</v>
@@ -12327,7 +12315,7 @@
         <v>2</v>
       </c>
       <c r="K100" t="n">
-        <v>26.8</v>
+        <v>27</v>
       </c>
       <c r="L100" t="n">
         <v>0</v>
@@ -12431,7 +12419,7 @@
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="n">
-        <v>0.8813559322033898</v>
+        <v>0.5</v>
       </c>
       <c r="G101" t="n">
         <v>0</v>
@@ -12446,7 +12434,7 @@
         <v>2</v>
       </c>
       <c r="K101" t="n">
-        <v>51.63461538461539</v>
+        <v>52</v>
       </c>
       <c r="L101" t="n">
         <v>0</v>
@@ -12669,7 +12657,7 @@
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="n">
-        <v>1.237373737373737</v>
+        <v>0.6186868686868687</v>
       </c>
       <c r="G103" t="n">
         <v>0</v>
@@ -12788,7 +12776,7 @@
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="n">
-        <v>4.347826086956522</v>
+        <v>0.4488498223302786</v>
       </c>
       <c r="G104" t="n">
         <v>0</v>
@@ -13026,7 +13014,7 @@
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="n">
-        <v>3.760204081632653</v>
+        <v>0.5537190082644629</v>
       </c>
       <c r="G106" t="n">
         <v>0</v>
@@ -13145,7 +13133,7 @@
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="n">
-        <v>25.20472727272728</v>
+        <v>0.6599143129165345</v>
       </c>
       <c r="G107" t="n">
         <v>0</v>
@@ -13264,7 +13252,7 @@
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="n">
-        <v>1.13265306122449</v>
+        <v>0.5080091533180778</v>
       </c>
       <c r="G108" t="n">
         <v>0</v>
@@ -13502,7 +13490,7 @@
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="n">
-        <v>1.536130536130536</v>
+        <v>0.4</v>
       </c>
       <c r="G110" t="n">
         <v>0</v>
@@ -13621,7 +13609,7 @@
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="n">
-        <v>0.4071246819338422</v>
+        <v>0.2182172430589381</v>
       </c>
       <c r="G111" t="n">
         <v>0</v>
@@ -13740,7 +13728,7 @@
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="n">
-        <v>1.099450274862569</v>
+        <v>0.5498625343664084</v>
       </c>
       <c r="G112" t="n">
         <v>0</v>
@@ -13859,7 +13847,7 @@
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="n">
-        <v>2.484429065743945</v>
+        <v>0.439717470297636</v>
       </c>
       <c r="G113" t="n">
         <v>0</v>
@@ -14097,7 +14085,7 @@
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="n">
-        <v>0.6269854539374686</v>
+        <v>0.2089951513124896</v>
       </c>
       <c r="G115" t="n">
         <v>0</v>
@@ -14112,7 +14100,7 @@
         <v>1</v>
       </c>
       <c r="K115" t="n">
-        <v>7.000000000000001</v>
+        <v>7</v>
       </c>
       <c r="L115" t="n">
         <v>0.15</v>
@@ -14216,7 +14204,7 @@
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="n">
-        <v>0.5936776708490681</v>
+        <v>0.1978925569496894</v>
       </c>
       <c r="G116" t="n">
         <v>0</v>
@@ -14231,7 +14219,7 @@
         <v>1</v>
       </c>
       <c r="K116" t="n">
-        <v>6.999999999999999</v>
+        <v>7</v>
       </c>
       <c r="L116" t="n">
         <v>0.15</v>
@@ -14335,7 +14323,7 @@
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G117" t="n">
         <v>0</v>
@@ -14454,7 +14442,7 @@
       <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="n">
-        <v>1.154285714285714</v>
+        <v>0.4</v>
       </c>
       <c r="G118" t="n">
         <v>0</v>
@@ -14573,7 +14561,7 @@
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="n">
-        <v>0.8660869565217391</v>
+        <v>0.4</v>
       </c>
       <c r="G119" t="n">
         <v>0</v>
@@ -14692,7 +14680,7 @@
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="n">
-        <v>0.6919191919191919</v>
+        <v>0.1548022598870057</v>
       </c>
       <c r="G120" t="n">
         <v>0</v>
@@ -14811,7 +14799,7 @@
       <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="n">
-        <v>0.28</v>
+        <v>0.2</v>
       </c>
       <c r="G121" t="n">
         <v>0</v>
@@ -14930,7 +14918,7 @@
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="n">
-        <v>0.3776041666666667</v>
+        <v>0.25</v>
       </c>
       <c r="G122" t="n">
         <v>0</v>
@@ -15168,7 +15156,7 @@
       <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="n">
-        <v>0.882706106870229</v>
+        <v>0.2856936380481779</v>
       </c>
       <c r="G124" t="n">
         <v>0</v>
@@ -15287,7 +15275,7 @@
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr"/>
       <c r="F125" t="n">
-        <v>0.8615384615384616</v>
+        <v>0.2572347266881029</v>
       </c>
       <c r="G125" t="n">
         <v>0</v>
@@ -15299,10 +15287,10 @@
         <v>0.07359675949418247</v>
       </c>
       <c r="J125" t="n">
-        <v>1.234267340376665</v>
+        <v>1</v>
       </c>
       <c r="K125" t="n">
-        <v>43.83096003674782</v>
+        <v>44</v>
       </c>
       <c r="L125" t="n">
         <v>0.09894350022967387</v>
@@ -15406,7 +15394,7 @@
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr"/>
       <c r="F126" t="n">
-        <v>0.8667447306791569</v>
+        <v>0.4469806763285025</v>
       </c>
       <c r="G126" t="n">
         <v>0</v>
@@ -15421,7 +15409,7 @@
         <v>1</v>
       </c>
       <c r="K126" t="n">
-        <v>25.71739130434782</v>
+        <v>26</v>
       </c>
       <c r="L126" t="n">
         <v>0.5616545893719807</v>
@@ -15525,7 +15513,7 @@
       <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="n">
-        <v>0.05981334249585128</v>
+        <v>0.01677926423000926</v>
       </c>
       <c r="G127" t="n">
         <v>0</v>
@@ -15644,7 +15632,7 @@
       <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr"/>
       <c r="F128" t="n">
-        <v>0.05509641873278237</v>
+        <v>0.04040404040404041</v>
       </c>
       <c r="G128" t="n">
         <v>0</v>
@@ -15763,7 +15751,7 @@
       <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr"/>
       <c r="F129" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="G129" t="n">
         <v>0</v>
@@ -15882,7 +15870,7 @@
       <c r="D130" t="inlineStr"/>
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="n">
-        <v>1.247165532879819</v>
+        <v>0.5386875612144956</v>
       </c>
       <c r="G130" t="n">
         <v>0</v>
@@ -15897,7 +15885,7 @@
         <v>1</v>
       </c>
       <c r="K130" t="n">
-        <v>27.43192948090108</v>
+        <v>27</v>
       </c>
       <c r="L130" t="n">
         <v>0.0455435847208619</v>
@@ -16001,7 +15989,7 @@
       <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr"/>
       <c r="F131" t="n">
-        <v>0.9306358381502891</v>
+        <v>0.3252525252525252</v>
       </c>
       <c r="G131" t="n">
         <v>0</v>
@@ -16016,7 +16004,7 @@
         <v>1</v>
       </c>
       <c r="K131" t="n">
-        <v>6.141414141414141</v>
+        <v>6</v>
       </c>
       <c r="L131" t="n">
         <v>0.4104040404040404</v>
@@ -16120,7 +16108,7 @@
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="n">
-        <v>2.666666666666667</v>
+        <v>0.3338549817423057</v>
       </c>
       <c r="G132" t="n">
         <v>0</v>
@@ -16239,7 +16227,7 @@
       <c r="D133" t="inlineStr"/>
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="n">
-        <v>1.052631578947368</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="G133" t="n">
         <v>0</v>
@@ -16254,7 +16242,7 @@
         <v>1</v>
       </c>
       <c r="K133" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="L133" t="n">
         <v>0.15</v>
@@ -16477,7 +16465,7 @@
       <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="n">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
       <c r="G135" t="n">
         <v>0</v>
@@ -16596,7 +16584,7 @@
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G136" t="n">
         <v>0</v>
@@ -16715,7 +16703,7 @@
       <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr"/>
       <c r="F137" t="n">
-        <v>0.7759036144578313</v>
+        <v>0.400497512437811</v>
       </c>
       <c r="G137" t="n">
         <v>0</v>
@@ -16834,7 +16822,7 @@
       <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="n">
-        <v>1.80948275862069</v>
+        <v>0.398292220113852</v>
       </c>
       <c r="G138" t="n">
         <v>0</v>
@@ -16953,7 +16941,7 @@
       <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="G139" t="n">
         <v>0</v>
@@ -17191,7 +17179,7 @@
       <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="n">
-        <v>2.839999999999999</v>
+        <v>0.4067369385884509</v>
       </c>
       <c r="G141" t="n">
         <v>0</v>
@@ -17206,7 +17194,7 @@
         <v>1</v>
       </c>
       <c r="K141" t="n">
-        <v>17.5627864344638</v>
+        <v>18</v>
       </c>
       <c r="L141" t="n">
         <v>0.15</v>
@@ -17429,7 +17417,7 @@
       <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr"/>
       <c r="F143" t="n">
-        <v>1.406779661016949</v>
+        <v>0.3802687843616371</v>
       </c>
       <c r="G143" t="n">
         <v>0</v>
@@ -17667,7 +17655,7 @@
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr"/>
       <c r="F145" t="n">
-        <v>0.5178571428571429</v>
+        <v>0.2589285714285715</v>
       </c>
       <c r="G145" t="n">
         <v>0</v>
@@ -17786,7 +17774,7 @@
       <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr"/>
       <c r="F146" t="n">
-        <v>1.328428927680798</v>
+        <v>0.5087870105062082</v>
       </c>
       <c r="G146" t="n">
         <v>0</v>
@@ -17905,7 +17893,7 @@
       <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="n">
-        <v>0.3206342728889148</v>
+        <v>0.2946928496798564</v>
       </c>
       <c r="G147" t="n">
         <v>0</v>
@@ -18024,7 +18012,7 @@
       <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr"/>
       <c r="F148" t="n">
-        <v>0.3533333333333333</v>
+        <v>0.175448275862069</v>
       </c>
       <c r="G148" t="n">
         <v>0</v>
@@ -18381,7 +18369,7 @@
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="n">
-        <v>0.2505454545454546</v>
+        <v>0.1093650793650794</v>
       </c>
       <c r="G151" t="n">
         <v>0</v>
@@ -18500,7 +18488,7 @@
       <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="n">
-        <v>0.1721854304635762</v>
+        <v>0.1660280970625798</v>
       </c>
       <c r="G152" t="n">
         <v>0</v>
@@ -18619,7 +18607,7 @@
       <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="n">
-        <v>0.326</v>
+        <v>0.1314516129032258</v>
       </c>
       <c r="G153" t="n">
         <v>0</v>
@@ -18738,7 +18726,7 @@
       <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr"/>
       <c r="F154" t="n">
-        <v>2.522151898734177</v>
+        <v>0.4027693551647463</v>
       </c>
       <c r="G154" t="n">
         <v>0</v>
@@ -18857,7 +18845,7 @@
       <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr"/>
       <c r="F155" t="n">
-        <v>0.3300247487762296</v>
+        <v>0.2785546766443466</v>
       </c>
       <c r="G155" t="n">
         <v>0</v>
@@ -18976,7 +18964,7 @@
       <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="n">
-        <v>0.9100434782608694</v>
+        <v>0.3564847142978795</v>
       </c>
       <c r="G156" t="n">
         <v>0</v>
@@ -19095,7 +19083,7 @@
       <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr"/>
       <c r="F157" t="n">
-        <v>0.275</v>
+        <v>0.2291666666666667</v>
       </c>
       <c r="G157" t="n">
         <v>0</v>
@@ -19214,7 +19202,7 @@
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr"/>
       <c r="F158" t="n">
-        <v>0.8479864636209813</v>
+        <v>0.3305804749340369</v>
       </c>
       <c r="G158" t="n">
         <v>0</v>
@@ -19333,7 +19321,7 @@
       <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr"/>
       <c r="F159" t="n">
-        <v>0.9235443037974682</v>
+        <v>0.4108108108108108</v>
       </c>
       <c r="G159" t="n">
         <v>0</v>
@@ -19348,7 +19336,7 @@
         <v>1</v>
       </c>
       <c r="K159" t="n">
-        <v>25.23423423423423</v>
+        <v>25</v>
       </c>
       <c r="L159" t="n">
         <v>0.15</v>
@@ -19452,7 +19440,7 @@
       <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr"/>
       <c r="F160" t="n">
-        <v>1.289288888888889</v>
+        <v>0.2732187426418649</v>
       </c>
       <c r="G160" t="n">
         <v>0</v>
@@ -19571,7 +19559,7 @@
       <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr"/>
       <c r="F161" t="n">
-        <v>0.4891462175112531</v>
+        <v>0.1043174657242613</v>
       </c>
       <c r="G161" t="n">
         <v>0</v>
@@ -19690,7 +19678,7 @@
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="n">
-        <v>7.059754797441364</v>
+        <v>0.3481717964046355</v>
       </c>
       <c r="G162" t="n">
         <v>0</v>
@@ -19705,7 +19693,7 @@
         <v>1</v>
       </c>
       <c r="K162" t="n">
-        <v>26.53332081985374</v>
+        <v>27</v>
       </c>
       <c r="L162" t="n">
         <v>0.15</v>
@@ -19928,7 +19916,7 @@
       <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="n">
-        <v>0.3078111540810348</v>
+        <v>0.2773569137777507</v>
       </c>
       <c r="G164" t="n">
         <v>0</v>
@@ -19943,7 +19931,7 @@
         <v>1</v>
       </c>
       <c r="K164" t="n">
-        <v>26.93879709910967</v>
+        <v>27</v>
       </c>
       <c r="L164" t="n">
         <v>0.15</v>
@@ -20047,7 +20035,7 @@
       <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr"/>
       <c r="F165" t="n">
-        <v>1.206666666666667</v>
+        <v>0.4087829360100376</v>
       </c>
       <c r="G165" t="n">
         <v>0</v>
@@ -20062,7 +20050,7 @@
         <v>1</v>
       </c>
       <c r="K165" t="n">
-        <v>23.83814303638645</v>
+        <v>24</v>
       </c>
       <c r="L165" t="n">
         <v>0.15</v>
@@ -20285,7 +20273,7 @@
       <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="n">
-        <v>0.08548387096774193</v>
+        <v>0.06309523809523809</v>
       </c>
       <c r="G167" t="n">
         <v>0</v>
@@ -20300,7 +20288,7 @@
         <v>1</v>
       </c>
       <c r="K167" t="n">
-        <v>23.33333333333333</v>
+        <v>23</v>
       </c>
       <c r="L167" t="n">
         <v>0.15</v>
@@ -20404,7 +20392,7 @@
       <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="n">
-        <v>0.4173333333333333</v>
+        <v>0.1399946327936309</v>
       </c>
       <c r="G168" t="n">
         <v>0</v>
@@ -20419,7 +20407,7 @@
         <v>1</v>
       </c>
       <c r="K168" t="n">
-        <v>24.0832811521603</v>
+        <v>24</v>
       </c>
       <c r="L168" t="n">
         <v>0.15</v>
@@ -20642,7 +20630,7 @@
       <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="n">
-        <v>1.840493827160494</v>
+        <v>0.4175278809367771</v>
       </c>
       <c r="G170" t="n">
         <v>0</v>
@@ -20761,7 +20749,7 @@
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr"/>
       <c r="F171" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.04450409720259961</v>
       </c>
       <c r="G171" t="n">
         <v>0</v>
@@ -20880,7 +20868,7 @@
       <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr"/>
       <c r="F172" t="n">
-        <v>0.9095842696629214</v>
+        <v>0.4390075921908894</v>
       </c>
       <c r="G172" t="n">
         <v>0</v>
@@ -21118,7 +21106,7 @@
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr"/>
       <c r="F174" t="n">
-        <v>1.377016129032258</v>
+        <v>0.6419172932330827</v>
       </c>
       <c r="G174" t="n">
         <v>0</v>
@@ -21475,7 +21463,7 @@
       <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr"/>
       <c r="F177" t="n">
-        <v>0.01923076923076923</v>
+        <v>0.01538461538461539</v>
       </c>
       <c r="G177" t="n">
         <v>0</v>
@@ -21713,7 +21701,7 @@
       <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr"/>
       <c r="F179" t="n">
-        <v>1.282101167315175</v>
+        <v>0.3655695266272189</v>
       </c>
       <c r="G179" t="n">
         <v>0</v>
@@ -21832,7 +21820,7 @@
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="n">
-        <v>0.3</v>
+        <v>0.1917747278936075</v>
       </c>
       <c r="G180" t="n">
         <v>0</v>
@@ -21951,7 +21939,7 @@
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="n">
-        <v>1.399333333333333</v>
+        <v>0.5879551820728292</v>
       </c>
       <c r="G181" t="n">
         <v>0</v>
@@ -22070,7 +22058,7 @@
       <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="n">
-        <v>2.077169811320755</v>
+        <v>0.6456891495601174</v>
       </c>
       <c r="G182" t="n">
         <v>0</v>
@@ -22189,7 +22177,7 @@
       <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr"/>
       <c r="F183" t="n">
-        <v>0.4690026954177898</v>
+        <v>0.4317617866004963</v>
       </c>
       <c r="G183" t="n">
         <v>0</v>
@@ -22308,7 +22296,7 @@
       <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr"/>
       <c r="F184" t="n">
-        <v>0.3305785123966942</v>
+        <v>0.1809954751131222</v>
       </c>
       <c r="G184" t="n">
         <v>0</v>
@@ -22546,7 +22534,7 @@
       <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr"/>
       <c r="F186" t="n">
-        <v>1.283636363636364</v>
+        <v>0.3519441674975075</v>
       </c>
       <c r="G186" t="n">
         <v>0</v>
@@ -22903,7 +22891,7 @@
       <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr"/>
       <c r="F189" t="n">
-        <v>0.116</v>
+        <v>0.04145818441744103</v>
       </c>
       <c r="G189" t="n">
         <v>0</v>
@@ -23022,7 +23010,7 @@
       <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr"/>
       <c r="F190" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G190" t="n">
         <v>0</v>
@@ -23260,7 +23248,7 @@
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="n">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="G192" t="n">
         <v>0</v>
@@ -23379,7 +23367,7 @@
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="G193" t="n">
         <v>0</v>
@@ -23617,7 +23605,7 @@
       <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr"/>
       <c r="F195" t="n">
-        <v>1.022765957446808</v>
+        <v>0.5253551912568306</v>
       </c>
       <c r="G195" t="n">
         <v>0</v>
@@ -23855,7 +23843,7 @@
       <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="n">
-        <v>0.8879240162822252</v>
+        <v>0.3505088377075522</v>
       </c>
       <c r="G197" t="n">
         <v>0</v>
@@ -23870,7 +23858,7 @@
         <v>1</v>
       </c>
       <c r="K197" t="n">
-        <v>15.02570969469738</v>
+        <v>15</v>
       </c>
       <c r="L197" t="n">
         <v>0.15</v>
@@ -23974,7 +23962,7 @@
       <c r="D198" t="inlineStr"/>
       <c r="E198" t="inlineStr"/>
       <c r="F198" t="n">
-        <v>1.446771428571429</v>
+        <v>0.3371304926764314</v>
       </c>
       <c r="G198" t="n">
         <v>0</v>
@@ -24093,7 +24081,7 @@
       <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="n">
-        <v>1.990253067484663</v>
+        <v>0.4113631320336028</v>
       </c>
       <c r="G199" t="n">
         <v>0</v>
@@ -24212,7 +24200,7 @@
       <c r="D200" t="inlineStr"/>
       <c r="E200" t="inlineStr"/>
       <c r="F200" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="G200" t="n">
         <v>0</v>
@@ -24569,7 +24557,7 @@
       <c r="D203" t="inlineStr"/>
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="n">
-        <v>0.1480645161290323</v>
+        <v>0.1136138613861386</v>
       </c>
       <c r="G203" t="n">
         <v>0</v>
@@ -24584,7 +24572,7 @@
         <v>1</v>
       </c>
       <c r="K203" t="n">
-        <v>13.48514851485148</v>
+        <v>13</v>
       </c>
       <c r="L203" t="n">
         <v>0.15</v>
@@ -24688,7 +24676,7 @@
       <c r="D204" t="inlineStr"/>
       <c r="E204" t="inlineStr"/>
       <c r="F204" t="n">
-        <v>0.2196902654867257</v>
+        <v>0.1948587127158556</v>
       </c>
       <c r="G204" t="n">
         <v>0</v>
@@ -24703,7 +24691,7 @@
         <v>1</v>
       </c>
       <c r="K204" t="n">
-        <v>2.843014128728414</v>
+        <v>3</v>
       </c>
       <c r="L204" t="n">
         <v>0.15</v>
@@ -25045,7 +25033,7 @@
       <c r="D207" t="inlineStr"/>
       <c r="E207" t="inlineStr"/>
       <c r="F207" t="n">
-        <v>2.823847566574839</v>
+        <v>0.3664996156436033</v>
       </c>
       <c r="G207" t="n">
         <v>0</v>
@@ -25402,7 +25390,7 @@
       <c r="D210" t="inlineStr"/>
       <c r="E210" t="inlineStr"/>
       <c r="F210" t="n">
-        <v>0.7956834532374101</v>
+        <v>0.3990378833433554</v>
       </c>
       <c r="G210" t="n">
         <v>0</v>
@@ -25521,7 +25509,7 @@
       <c r="D211" t="inlineStr"/>
       <c r="E211" t="inlineStr"/>
       <c r="F211" t="n">
-        <v>1.252897670824594</v>
+        <v>0.2225155100420952</v>
       </c>
       <c r="G211" t="n">
         <v>0</v>
@@ -25533,10 +25521,10 @@
         <v>0.02844200129694474</v>
       </c>
       <c r="J211" t="n">
-        <v>0.389083465074483</v>
+        <v>0</v>
       </c>
       <c r="K211" t="n">
-        <v>8.170752766564142</v>
+        <v>8</v>
       </c>
       <c r="L211" t="n">
         <v>0.15</v>
@@ -25759,7 +25747,7 @@
       <c r="D213" t="inlineStr"/>
       <c r="E213" t="inlineStr"/>
       <c r="F213" t="n">
-        <v>2.452242609582059</v>
+        <v>0.5414626989661129</v>
       </c>
       <c r="G213" t="n">
         <v>0</v>
@@ -25878,7 +25866,7 @@
       <c r="D214" t="inlineStr"/>
       <c r="E214" t="inlineStr"/>
       <c r="F214" t="n">
-        <v>8.683190913433469</v>
+        <v>1.460062472110665</v>
       </c>
       <c r="G214" t="n">
         <v>0</v>
@@ -25997,7 +25985,7 @@
       <c r="D215" t="inlineStr"/>
       <c r="E215" t="inlineStr"/>
       <c r="F215" t="n">
-        <v>6.662983425414365</v>
+        <v>0.489746192893401</v>
       </c>
       <c r="G215" t="n">
         <v>0</v>
@@ -26116,7 +26104,7 @@
       <c r="D216" t="inlineStr"/>
       <c r="E216" t="inlineStr"/>
       <c r="F216" t="n">
-        <v>0.9513444302176697</v>
+        <v>0.4687697160883281</v>
       </c>
       <c r="G216" t="n">
         <v>0</v>
@@ -26235,7 +26223,7 @@
       <c r="D217" t="inlineStr"/>
       <c r="E217" t="inlineStr"/>
       <c r="F217" t="n">
-        <v>3.659737156511351</v>
+        <v>0.4000000000000001</v>
       </c>
       <c r="G217" t="n">
         <v>0</v>
@@ -26473,7 +26461,7 @@
       <c r="D219" t="inlineStr"/>
       <c r="E219" t="inlineStr"/>
       <c r="F219" t="n">
-        <v>0.6360606060606061</v>
+        <v>0.2931122121244282</v>
       </c>
       <c r="G219" t="n">
         <v>0</v>
@@ -26488,7 +26476,7 @@
         <v>1</v>
       </c>
       <c r="K219" t="n">
-        <v>26.96187725873751</v>
+        <v>27</v>
       </c>
       <c r="L219" t="n">
         <v>0.15</v>
@@ -26604,7 +26592,7 @@
         <v>0.04</v>
       </c>
       <c r="J220" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="K220" t="n">
         <v>27</v>
@@ -26830,7 +26818,7 @@
       <c r="D222" t="inlineStr"/>
       <c r="E222" t="inlineStr"/>
       <c r="F222" t="n">
-        <v>1.105268385174484</v>
+        <v>0.3404455321634174</v>
       </c>
       <c r="G222" t="n">
         <v>0</v>
@@ -26842,7 +26830,7 @@
         <v>0.06706788664237839</v>
       </c>
       <c r="J222" t="n">
-        <v>3.909725505464861</v>
+        <v>4</v>
       </c>
       <c r="K222" t="n">
         <v>27</v>
@@ -27068,7 +27056,7 @@
       <c r="D224" t="inlineStr"/>
       <c r="E224" t="inlineStr"/>
       <c r="F224" t="n">
-        <v>1.667832167832168</v>
+        <v>0.5585480093676815</v>
       </c>
       <c r="G224" t="n">
         <v>0</v>
@@ -27083,7 +27071,7 @@
         <v>4</v>
       </c>
       <c r="K224" t="n">
-        <v>20.28337236533958</v>
+        <v>20</v>
       </c>
       <c r="L224" t="n">
         <v>0.15</v>
@@ -27306,7 +27294,7 @@
       <c r="D226" t="inlineStr"/>
       <c r="E226" t="inlineStr"/>
       <c r="F226" t="n">
-        <v>0.7100000000000001</v>
+        <v>0.2561635598316296</v>
       </c>
       <c r="G226" t="n">
         <v>0</v>
@@ -27321,7 +27309,7 @@
         <v>1</v>
       </c>
       <c r="K226" t="n">
-        <v>13.11725796752856</v>
+        <v>13</v>
       </c>
       <c r="L226" t="n">
         <v>0.15</v>
@@ -27425,7 +27413,7 @@
       <c r="D227" t="inlineStr"/>
       <c r="E227" t="inlineStr"/>
       <c r="F227" t="n">
-        <v>0.8632520325203252</v>
+        <v>0.2902679059595407</v>
       </c>
       <c r="G227" t="n">
         <v>0</v>
@@ -27544,7 +27532,7 @@
       <c r="D228" t="inlineStr"/>
       <c r="E228" t="inlineStr"/>
       <c r="F228" t="n">
-        <v>1.090909090909091</v>
+        <v>0.5504587155963303</v>
       </c>
       <c r="G228" t="n">
         <v>0</v>
@@ -27556,7 +27544,7 @@
         <v>0.005045871559633028</v>
       </c>
       <c r="J228" t="n">
-        <v>0.5045871559633027</v>
+        <v>1</v>
       </c>
       <c r="K228" t="n">
         <v>26</v>
@@ -27782,7 +27770,7 @@
       <c r="D230" t="inlineStr"/>
       <c r="E230" t="inlineStr"/>
       <c r="F230" t="n">
-        <v>4.99672131147541</v>
+        <v>0.7377022993657891</v>
       </c>
       <c r="G230" t="n">
         <v>0</v>
@@ -27794,10 +27782,10 @@
         <v>0.04634190371726445</v>
       </c>
       <c r="J230" t="n">
-        <v>1.540097798800895</v>
+        <v>2</v>
       </c>
       <c r="K230" t="n">
-        <v>31.97966768544452</v>
+        <v>32</v>
       </c>
       <c r="L230" t="n">
         <v>0</v>
@@ -27901,7 +27889,7 @@
       <c r="D231" t="inlineStr"/>
       <c r="E231" t="inlineStr"/>
       <c r="F231" t="n">
-        <v>1.311475409836065</v>
+        <v>0.6557377049180327</v>
       </c>
       <c r="G231" t="n">
         <v>0</v>
@@ -27913,7 +27901,7 @@
         <v>0.0385</v>
       </c>
       <c r="J231" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="K231" t="n">
         <v>27</v>
@@ -28020,7 +28008,7 @@
       <c r="D232" t="inlineStr"/>
       <c r="E232" t="inlineStr"/>
       <c r="F232" t="n">
-        <v>0.5171428571428572</v>
+        <v>0.4022222222222223</v>
       </c>
       <c r="G232" t="n">
         <v>0</v>
@@ -28139,7 +28127,7 @@
       <c r="D233" t="inlineStr"/>
       <c r="E233" t="inlineStr"/>
       <c r="F233" t="n">
-        <v>1.994571428571429</v>
+        <v>0.4</v>
       </c>
       <c r="G233" t="n">
         <v>0</v>
@@ -28377,7 +28365,7 @@
       <c r="D235" t="inlineStr"/>
       <c r="E235" t="inlineStr"/>
       <c r="F235" t="n">
-        <v>0.6155236458565186</v>
+        <v>0.4000000000000001</v>
       </c>
       <c r="G235" t="n">
         <v>0</v>
@@ -28496,7 +28484,7 @@
       <c r="D236" t="inlineStr"/>
       <c r="E236" t="inlineStr"/>
       <c r="F236" t="n">
-        <v>0.08928571428571429</v>
+        <v>0.03311258278145696</v>
       </c>
       <c r="G236" t="n">
         <v>0</v>
@@ -28615,7 +28603,7 @@
       <c r="D237" t="inlineStr"/>
       <c r="E237" t="inlineStr"/>
       <c r="F237" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="G237" t="n">
         <v>0</v>
@@ -28972,7 +28960,7 @@
       <c r="D240" t="inlineStr"/>
       <c r="E240" t="inlineStr"/>
       <c r="F240" t="n">
-        <v>1.046816479400749</v>
+        <v>0.2547857793983592</v>
       </c>
       <c r="G240" t="n">
         <v>0</v>
@@ -28987,7 +28975,7 @@
         <v>1</v>
       </c>
       <c r="K240" t="n">
-        <v>15.22060164083865</v>
+        <v>15</v>
       </c>
       <c r="L240" t="n">
         <v>0.15</v>
@@ -29210,7 +29198,7 @@
       <c r="D242" t="inlineStr"/>
       <c r="E242" t="inlineStr"/>
       <c r="F242" t="n">
-        <v>0.7859306596847524</v>
+        <v>0.51928382223574</v>
       </c>
       <c r="G242" t="n">
         <v>0</v>
@@ -29567,7 +29555,7 @@
       <c r="D245" t="inlineStr"/>
       <c r="E245" t="inlineStr"/>
       <c r="F245" t="n">
-        <v>0.6283798821919208</v>
+        <v>0.4737889219230008</v>
       </c>
       <c r="G245" t="n">
         <v>0</v>
@@ -29582,7 +29570,7 @@
         <v>1</v>
       </c>
       <c r="K245" t="n">
-        <v>19.46015132963318</v>
+        <v>19</v>
       </c>
       <c r="L245" t="n">
         <v>0</v>
@@ -29805,7 +29793,7 @@
       <c r="D247" t="inlineStr"/>
       <c r="E247" t="inlineStr"/>
       <c r="F247" t="n">
-        <v>0.5700019718778602</v>
+        <v>0.1920539842731593</v>
       </c>
       <c r="G247" t="n">
         <v>0</v>
@@ -29817,7 +29805,7 @@
         <v>0.05614809624121472</v>
       </c>
       <c r="J247" t="n">
-        <v>0.9353265211723645</v>
+        <v>1</v>
       </c>
       <c r="K247" t="n">
         <v>27</v>
@@ -29924,7 +29912,7 @@
       <c r="D248" t="inlineStr"/>
       <c r="E248" t="inlineStr"/>
       <c r="F248" t="n">
-        <v>0.3587452167292876</v>
+        <v>0.1931788814193691</v>
       </c>
       <c r="G248" t="n">
         <v>0</v>
@@ -29936,7 +29924,7 @@
         <v>0.09256926603565364</v>
       </c>
       <c r="J248" t="n">
-        <v>0.6222987310251633</v>
+        <v>1</v>
       </c>
       <c r="K248" t="n">
         <v>27</v>
@@ -30400,7 +30388,7 @@
       <c r="D252" t="inlineStr"/>
       <c r="E252" t="inlineStr"/>
       <c r="F252" t="n">
-        <v>0.1439642656688494</v>
+        <v>0.1237538397208061</v>
       </c>
       <c r="G252" t="n">
         <v>0</v>
@@ -30412,7 +30400,7 @@
         <v>0.09730596089460676</v>
       </c>
       <c r="J252" t="n">
-        <v>1.859614982550379</v>
+        <v>2</v>
       </c>
       <c r="K252" t="n">
         <v>27</v>
@@ -30757,7 +30745,7 @@
       <c r="D255" t="inlineStr"/>
       <c r="E255" t="inlineStr"/>
       <c r="F255" t="n">
-        <v>4.967730561184984</v>
+        <v>0.844</v>
       </c>
       <c r="G255" t="n">
         <v>0</v>
@@ -30769,7 +30757,7 @@
         <v>0.01158772435000062</v>
       </c>
       <c r="J255" t="n">
-        <v>2.341245915880973</v>
+        <v>2</v>
       </c>
       <c r="K255" t="n">
         <v>18</v>
@@ -30876,7 +30864,7 @@
       <c r="D256" t="inlineStr"/>
       <c r="E256" t="inlineStr"/>
       <c r="F256" t="n">
-        <v>0.9759162303664923</v>
+        <v>0.4000000000000001</v>
       </c>
       <c r="G256" t="n">
         <v>0</v>
@@ -30995,7 +30983,7 @@
       <c r="D257" t="inlineStr"/>
       <c r="E257" t="inlineStr"/>
       <c r="F257" t="n">
-        <v>33.36101265822784</v>
+        <v>0.4</v>
       </c>
       <c r="G257" t="n">
         <v>0</v>
@@ -31114,7 +31102,7 @@
       <c r="D258" t="inlineStr"/>
       <c r="E258" t="inlineStr"/>
       <c r="F258" t="n">
-        <v>3.528981233243969</v>
+        <v>0.2</v>
       </c>
       <c r="G258" t="n">
         <v>0</v>
@@ -31233,7 +31221,7 @@
       <c r="D259" t="inlineStr"/>
       <c r="E259" t="inlineStr"/>
       <c r="F259" t="n">
-        <v>5.028827701293284</v>
+        <v>0.2</v>
       </c>
       <c r="G259" t="n">
         <v>0</v>
@@ -31352,7 +31340,7 @@
       <c r="D260" t="inlineStr"/>
       <c r="E260" t="inlineStr"/>
       <c r="F260" t="n">
-        <v>1.248458149779736</v>
+        <v>0.5</v>
       </c>
       <c r="G260" t="n">
         <v>0</v>
@@ -31471,7 +31459,7 @@
       <c r="D261" t="inlineStr"/>
       <c r="E261" t="inlineStr"/>
       <c r="F261" t="n">
-        <v>0.6174112256586484</v>
+        <v>0.5</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
@@ -31590,7 +31578,7 @@
       <c r="D262" t="inlineStr"/>
       <c r="E262" t="inlineStr"/>
       <c r="F262" t="n">
-        <v>0.943089430894309</v>
+        <v>0.4</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
@@ -31709,7 +31697,7 @@
       <c r="D263" t="inlineStr"/>
       <c r="E263" t="inlineStr"/>
       <c r="F263" t="n">
-        <v>8.669724770642201</v>
+        <v>0.5</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
@@ -31828,7 +31816,7 @@
       <c r="D264" t="inlineStr"/>
       <c r="E264" t="inlineStr"/>
       <c r="F264" t="n">
-        <v>1.17479674796748</v>
+        <v>0.4873524451939292</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
@@ -32066,7 +32054,7 @@
       <c r="D266" t="inlineStr"/>
       <c r="E266" t="inlineStr"/>
       <c r="F266" t="n">
-        <v>1.10126582278481</v>
+        <v>0.2230769230769231</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
@@ -32304,7 +32292,7 @@
       <c r="D268" t="inlineStr"/>
       <c r="E268" t="inlineStr"/>
       <c r="F268" t="n">
-        <v>0.8228571428571428</v>
+        <v>0.4114285714285714</v>
       </c>
       <c r="G268" t="n">
         <v>0</v>
@@ -32423,7 +32411,7 @@
       <c r="D269" t="inlineStr"/>
       <c r="E269" t="inlineStr"/>
       <c r="F269" t="n">
-        <v>0.09375</v>
+        <v>0.07894736842105263</v>
       </c>
       <c r="G269" t="n">
         <v>0</v>
@@ -32438,7 +32426,7 @@
         <v>1</v>
       </c>
       <c r="K269" t="n">
-        <v>14.26315789473684</v>
+        <v>14</v>
       </c>
       <c r="L269" t="n">
         <v>0.15</v>

</xml_diff>

<commit_message>
refactor: update parsing logic add new method to handle biomass-specific NET_MIN_STAB_GEN calculation to ensure min_stable_gen is within 0-1 range
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/thermal/specific_2030.xlsx
+++ b/tests/antares/resources/expected_output_files/thermal/specific_2030.xlsx
@@ -8740,7 +8740,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>0.6441778079144341</v>
+        <v>0.5</v>
       </c>
       <c r="D72" t="n">
         <v>0</v>
@@ -8856,7 +8856,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.741070105231955</v>
+        <v>0.5</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
@@ -9436,7 +9436,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>7.366482504604051</v>
+        <v>0.4</v>
       </c>
       <c r="D78" t="n">
         <v>0</v>
@@ -9552,7 +9552,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.3168839551847534</v>
+        <v>0.3161111226228085</v>
       </c>
       <c r="D79" t="n">
         <v>0</v>
@@ -10132,7 +10132,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1.568228210568039</v>
+        <v>0.5</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -10248,7 +10248,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0.6134758535539871</v>
+        <v>0.5</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>0.7352941176470589</v>
+        <v>0.3676470588235294</v>
       </c>
       <c r="D88" t="n">
         <v>0</v>
@@ -10712,7 +10712,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>0.7352941176470589</v>
+        <v>0.3676470588235294</v>
       </c>
       <c r="D89" t="n">
         <v>0</v>
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>0.8311688311688311</v>
+        <v>0.4</v>
       </c>
       <c r="D96" t="n">
         <v>0</v>
@@ -11640,7 +11640,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>0.6678989525569933</v>
+        <v>0.3958923803655782</v>
       </c>
       <c r="D97" t="n">
         <v>0</v>
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>0.2225155100420952</v>
+        <v>0.2128816667262639</v>
       </c>
       <c r="D211" t="n">
         <v>0</v>
@@ -24980,7 +24980,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1.624658708847621</v>
+        <v>0.7392197125256674</v>
       </c>
       <c r="D212" t="n">
         <v>0</v>
@@ -25096,7 +25096,7 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>0.5414626989661129</v>
+        <v>0.465054932907864</v>
       </c>
       <c r="D213" t="n">
         <v>0</v>
@@ -25212,7 +25212,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1.460062472110665</v>
+        <v>0.605925925925926</v>
       </c>
       <c r="D214" t="n">
         <v>0</v>
@@ -28460,7 +28460,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>0.51928382223574</v>
+        <v>0.3602285236087067</v>
       </c>
       <c r="D242" t="n">
         <v>0</v>
@@ -28576,7 +28576,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>0.1775110245694023</v>
+        <v>0.1373</v>
       </c>
       <c r="D243" t="n">
         <v>0</v>
@@ -29272,7 +29272,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>0.09037037037037036</v>
+        <v>0.0183</v>
       </c>
       <c r="D249" t="n">
         <v>0</v>
@@ -29388,7 +29388,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>0.02294670846394984</v>
+        <v>0.0183</v>
       </c>
       <c r="D250" t="n">
         <v>0</v>
@@ -29620,7 +29620,7 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>0.1237538397208061</v>
+        <v>0.0751652792743531</v>
       </c>
       <c r="D252" t="n">
         <v>0</v>
@@ -29736,7 +29736,7 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>0.4580701754385966</v>
+        <v>0.2611</v>
       </c>
       <c r="D253" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
refactor: update parsing and output file generation for specific thermal parameters NET_MIN_STAB_GEN
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/thermal/specific_2030.xlsx
+++ b/tests/antares/resources/expected_output_files/thermal/specific_2030.xlsx
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1416577903397606</v>
+        <v>0.5</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.1990984060954279</v>
+        <v>0.3452348312627042</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -2360,7 +2360,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.2364559819413093</v>
+        <v>0.3594808126410835</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -3636,7 +3636,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -3752,7 +3752,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -6304,7 +6304,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.2466414609414088</v>
+        <v>0.2471099054771444</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -6884,7 +6884,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0.3136308392817405</v>
+        <v>0.3209486639620671</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
@@ -7580,7 +7580,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0.1833030995515977</v>
+        <v>0.1941008787429029</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -8392,7 +8392,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.1148377688662049</v>
+        <v>0.2812613926358002</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
@@ -9784,7 +9784,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.4438652766639936</v>
+        <v>0.5</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
@@ -10364,7 +10364,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D86" t="n">
         <v>0</v>
@@ -12568,7 +12568,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
@@ -13612,7 +13612,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D114" t="n">
         <v>0</v>
@@ -14308,7 +14308,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>0.1548022598870057</v>
+        <v>0.2</v>
       </c>
       <c r="D120" t="n">
         <v>0</v>
@@ -15120,7 +15120,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>0.01677926423000926</v>
+        <v>0.2076438870381153</v>
       </c>
       <c r="D127" t="n">
         <v>0</v>
@@ -16860,7 +16860,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D142" t="n">
         <v>0</v>
@@ -17440,7 +17440,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>0.2946928496798564</v>
+        <v>0.3108741661531867</v>
       </c>
       <c r="D147" t="n">
         <v>0</v>
@@ -17556,7 +17556,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>0.175448275862069</v>
+        <v>0.1768275862068966</v>
       </c>
       <c r="D148" t="n">
         <v>0</v>
@@ -17904,7 +17904,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>0.1093650793650794</v>
+        <v>0.3911111111111111</v>
       </c>
       <c r="D151" t="n">
         <v>0</v>
@@ -18020,7 +18020,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>0.1660280970625798</v>
+        <v>0.1803320561941252</v>
       </c>
       <c r="D152" t="n">
         <v>0</v>
@@ -18136,7 +18136,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>0.1314516129032258</v>
+        <v>0.2524193548387097</v>
       </c>
       <c r="D153" t="n">
         <v>0</v>
@@ -18600,7 +18600,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>0.2291666666666667</v>
+        <v>0.3125</v>
       </c>
       <c r="D157" t="n">
         <v>0</v>
@@ -19064,7 +19064,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>0.1043174657242613</v>
+        <v>0.4794848768705535</v>
       </c>
       <c r="D161" t="n">
         <v>0</v>
@@ -19180,7 +19180,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>0.3481717964046355</v>
+        <v>0.3513264551257684</v>
       </c>
       <c r="D162" t="n">
         <v>0</v>
@@ -19412,7 +19412,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>0.2773569137777507</v>
+        <v>0.2865731168403916</v>
       </c>
       <c r="D164" t="n">
         <v>0</v>
@@ -19528,7 +19528,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>0.4087829360100376</v>
+        <v>0.4230865746549561</v>
       </c>
       <c r="D165" t="n">
         <v>0</v>
@@ -19876,7 +19876,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>0.1399946327936309</v>
+        <v>0.1735396726004115</v>
       </c>
       <c r="D168" t="n">
         <v>0</v>
@@ -20224,7 +20224,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>0.04450409720259961</v>
+        <v>0.2115004238485448</v>
       </c>
       <c r="D171" t="n">
         <v>0</v>
@@ -20572,7 +20572,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>0.6419172932330827</v>
+        <v>0.6644736842105263</v>
       </c>
       <c r="D174" t="n">
         <v>0</v>
@@ -20920,7 +20920,7 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>0.01538461538461539</v>
+        <v>0.4153846153846154</v>
       </c>
       <c r="D177" t="n">
         <v>0</v>
@@ -21268,7 +21268,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>0.1917747278936075</v>
+        <v>0.2639249092978692</v>
       </c>
       <c r="D180" t="n">
         <v>0</v>
@@ -21732,7 +21732,7 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>0.1809954751131222</v>
+        <v>0.2904977375565611</v>
       </c>
       <c r="D184" t="n">
         <v>0</v>
@@ -21848,7 +21848,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D185" t="n">
         <v>0</v>
@@ -24516,7 +24516,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D208" t="n">
         <v>0</v>
@@ -24632,7 +24632,7 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D209" t="n">
         <v>0</v>
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>0.2128816667262639</v>
+        <v>0.4572482806964707</v>
       </c>
       <c r="D211" t="n">
         <v>0</v>
@@ -25676,7 +25676,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D218" t="n">
         <v>0</v>
@@ -25792,7 +25792,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>0.2931122121244282</v>
+        <v>0.294680690622085</v>
       </c>
       <c r="D219" t="n">
         <v>0</v>
@@ -28692,7 +28692,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D244" t="n">
         <v>0</v>
@@ -30084,7 +30084,7 @@
         </is>
       </c>
       <c r="C256" t="n">
-        <v>0.4000000000000001</v>
+        <v>0</v>
       </c>
       <c r="D256" t="n">
         <v>0</v>
@@ -31592,7 +31592,7 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>0.07894736842105263</v>
+        <v>0.5</v>
       </c>
       <c r="D269" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
refactor(minor): parsing TS from param modulation updated to avoid pytes performance warning with pandas test expected files updated with new min values from TS param modulation
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/thermal/specific_2030.xlsx
+++ b/tests/antares/resources/expected_output_files/thermal/specific_2030.xlsx
@@ -5144,7 +5144,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.2</v>
+        <v>0.133</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
@@ -5260,7 +5260,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.4466083399735535</v>
+        <v>0.409</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
@@ -8856,7 +8856,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.5</v>
+        <v>0.265</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
@@ -9436,7 +9436,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>0.4</v>
+        <v>0.265</v>
       </c>
       <c r="D78" t="n">
         <v>0</v>
@@ -10132,7 +10132,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0.5</v>
+        <v>0.276</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -10248,7 +10248,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0.5</v>
+        <v>0.27</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
@@ -10364,7 +10364,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="D86" t="n">
         <v>0</v>
@@ -10828,7 +10828,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>0.5</v>
+        <v>0.238</v>
       </c>
       <c r="D90" t="n">
         <v>0</v>
@@ -12568,7 +12568,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>0.2</v>
+        <v>0.136</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
@@ -12800,7 +12800,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>0.6599143129165345</v>
+        <v>0.653</v>
       </c>
       <c r="D107" t="n">
         <v>0</v>
@@ -20804,7 +20804,7 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>0.3658536585365854</v>
+        <v>0.3</v>
       </c>
       <c r="D176" t="n">
         <v>0</v>
@@ -24516,7 +24516,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>0.4</v>
+        <v>0.274</v>
       </c>
       <c r="D208" t="n">
         <v>0</v>
@@ -25676,7 +25676,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>0.5</v>
+        <v>0.301</v>
       </c>
       <c r="D218" t="n">
         <v>0</v>
@@ -28344,7 +28344,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>0.1667</v>
+        <v>0</v>
       </c>
       <c r="D241" t="n">
         <v>0</v>
@@ -28460,7 +28460,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>0.3602285236087067</v>
+        <v>0</v>
       </c>
       <c r="D242" t="n">
         <v>0</v>
@@ -28576,7 +28576,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>0.1373</v>
+        <v>0</v>
       </c>
       <c r="D243" t="n">
         <v>0</v>
@@ -28692,7 +28692,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>0.5</v>
+        <v>0.373</v>
       </c>
       <c r="D244" t="n">
         <v>0</v>
@@ -28924,7 +28924,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D246" t="n">
         <v>0</v>
@@ -29040,7 +29040,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>0.1920539842731593</v>
+        <v>0.174</v>
       </c>
       <c r="D247" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
minor fix: update min_stable calculation to handle zero values and improve readability
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/thermal/specific_2030.xlsx
+++ b/tests/antares/resources/expected_output_files/thermal/specific_2030.xlsx
@@ -28344,7 +28344,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>0</v>
+        <v>0.1667</v>
       </c>
       <c r="D241" t="n">
         <v>0</v>
@@ -28460,7 +28460,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>0</v>
+        <v>0.3602285236087067</v>
       </c>
       <c r="D242" t="n">
         <v>0</v>
@@ -28576,7 +28576,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>0</v>
+        <v>0.1373</v>
       </c>
       <c r="D243" t="n">
         <v>0</v>
@@ -28924,7 +28924,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D246" t="n">
         <v>0</v>

</xml_diff>